<commit_message>
Restore user's loss-provision reversal direction (opening entry already credits provision)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011perRKT2EmENmrFmt59Nd9
</commit_message>
<xml_diff>
--- a/BIM分錄_Final_檢核版.xlsx
+++ b/BIM分錄_Final_檢核版.xlsx
@@ -3153,11 +3153,11 @@
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>55110006</v>
+        <v>25600020</v>
       </c>
       <c r="E29" s="143" t="inlineStr">
         <is>
-          <t>成本-負債準備</t>
+          <t>負債準備</t>
         </is>
       </c>
       <c r="F29" s="143">
@@ -3171,11 +3171,11 @@
         </is>
       </c>
       <c r="I29" s="8" t="n">
-        <v>55110006</v>
+        <v>25600020</v>
       </c>
       <c r="J29" s="143" t="inlineStr">
         <is>
-          <t>成本-負債準備</t>
+          <t>負債準備</t>
         </is>
       </c>
       <c r="K29" s="143">
@@ -3203,11 +3203,11 @@
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>25600020</v>
+        <v>55110006</v>
       </c>
       <c r="E30" s="143" t="inlineStr">
         <is>
-          <t>負債準備</t>
+          <t>成本-負債準備</t>
         </is>
       </c>
       <c r="F30" s="143">
@@ -3221,11 +3221,11 @@
         </is>
       </c>
       <c r="I30" s="8" t="n">
-        <v>25600020</v>
+        <v>55110006</v>
       </c>
       <c r="J30" s="143" t="inlineStr">
         <is>
-          <t>負債準備</t>
+          <t>成本-負債準備</t>
         </is>
       </c>
       <c r="K30" s="143">
@@ -5676,7 +5676,7 @@
       <c r="C81" s="14" t="n"/>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>本月提列虧損準備(虧損專案)</t>
+          <t>本月迴轉負債準備(虧損專案，開帳已提列)</t>
         </is>
       </c>
       <c r="E81" s="24" t="n">
@@ -6248,7 +6248,7 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>5 虧損專案（負債準備）（第29-30列）</t>
+          <t>5 虧損專案－迴轉負債準備（第29-30列）</t>
         </is>
       </c>
       <c r="B9" s="171">
@@ -7369,7 +7369,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="H29">
+      <c r="H29" s="0">
         <f>IF(工作表1!D29="","",LEFT(工作表1!D29,1))</f>
         <v/>
       </c>
@@ -7381,7 +7381,7 @@
         <f>IF(工作表1!D29="",0,IF(COUNTIF(工作表1!$C$52:$C$71,工作表1!D29)&gt;0,0,1))</f>
         <v/>
       </c>
-      <c r="K29">
+      <c r="K29" s="0">
         <f>IF(工作表1!I29="","",LEFT(工作表1!I29,1))</f>
         <v/>
       </c>
@@ -7393,7 +7393,7 @@
         <f>IF(工作表1!I29="",0,IF(COUNTIF(工作表1!$H$52:$H$71,工作表1!I29)&gt;0,0,1))</f>
         <v/>
       </c>
-      <c r="N29">
+      <c r="N29" s="0">
         <f>IF(工作表1!N29="","",LEFT(工作表1!N29,1))</f>
         <v/>
       </c>
@@ -7405,7 +7405,7 @@
         <f>IF(工作表1!N29="",0,IF(COUNTIF(工作表1!$M$52:$M$71,工作表1!N29)&gt;0,0,1))</f>
         <v/>
       </c>
-      <c r="Q29">
+      <c r="Q29" s="0">
         <f>IF(工作表1!S29="","",LEFT(工作表1!S29,1))</f>
         <v/>
       </c>
@@ -7419,7 +7419,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="H30">
+      <c r="H30" s="0">
         <f>IF(工作表1!D30="","",LEFT(工作表1!D30,1))</f>
         <v/>
       </c>
@@ -7431,7 +7431,7 @@
         <f>IF(工作表1!D30="",0,IF(COUNTIF(工作表1!$C$52:$C$71,工作表1!D30)&gt;0,0,1))</f>
         <v/>
       </c>
-      <c r="K30">
+      <c r="K30" s="0">
         <f>IF(工作表1!I30="","",LEFT(工作表1!I30,1))</f>
         <v/>
       </c>
@@ -7443,7 +7443,7 @@
         <f>IF(工作表1!I30="",0,IF(COUNTIF(工作表1!$H$52:$H$71,工作表1!I30)&gt;0,0,1))</f>
         <v/>
       </c>
-      <c r="N30">
+      <c r="N30" s="0">
         <f>IF(工作表1!N30="","",LEFT(工作表1!N30,1))</f>
         <v/>
       </c>
@@ -7455,7 +7455,7 @@
         <f>IF(工作表1!N30="",0,IF(COUNTIF(工作表1!$M$52:$M$71,工作表1!N30)&gt;0,0,1))</f>
         <v/>
       </c>
-      <c r="Q30">
+      <c r="Q30" s="0">
         <f>IF(工作表1!S30="","",LEFT(工作表1!S30,1))</f>
         <v/>
       </c>

</xml_diff>